<commit_message>
B&N rev5: audit rev4 applied, back-check comments resolved (fire stop track 264.21 LF), all gates OK
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/FINAL_FOR_REVIEW_2026-10-24_rev5/Take-off/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev5.xlsx
+++ b/cache_proyectos/barnes_noble/FINAL_FOR_REVIEW_2026-10-24_rev5/Take-off/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev5.xlsx
@@ -1054,7 +1054,7 @@
     <t xml:space="preserve">Track, ceilings / soffits / canopy</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: 2/A-221, 3/A-221, 6/A-210, 4/A-210, 8/A-410, 5/A-121 | Breakdown [DERIVED]: SS-N 45.54 + SS-E 20.24 + SS-IN-N 40 + SS-IN-E 12.5 + SS-GG 12.33 + Women's Restroom 109 32.33 + Men's Restroom 108 32.33 + Cafe 103 - 11'-6" GWB band 52.51 + Cafe 103 - 9'-0" GWB band 43.33 + VEST-BOX-BEAM-TRACK 25.33 + VEST-LEDGER 12.67 + VEST-POSTS-TRACK 5 + FIRESTOP-TRACK-3 142.74 + FIRESTOP-TRACK-6 87.4 = 564.25 LF</t>
+    <t xml:space="preserve">N/SHEET: 2/A-221, 3/A-221, 6/A-210, 4/A-210, 8/A-410, 5/A-121 | Breakdown [DERIVED]: SS-N 45.54 + SS-E 20.24 + SS-IN-N 40 + SS-IN-E 12.5 + SS-GG 12.33 + Women's Restroom 109 32.33 + Men's Restroom 108 32.33 + Cafe 103 - 11'-6" GWB band 52.51 + Cafe 103 - 9'-0" GWB band 43.33 + VEST-BOX-BEAM-TRACK 25.33 + VEST-LEDGER 12.67 + VEST-POSTS-TRACK 5 + FIRESTOP-TRACK-3 157.81 + FIRESTOP-TRACK-6 106.4 = 598.32 LF</t>
   </si>
   <si>
     <t xml:space="preserve">Bracing 1-1/2" C.R. channel @ 48" O.C.</t>
@@ -1123,7 +1123,7 @@
     <t xml:space="preserve">USG drywall suspension main tee DGLW26</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: 4/A-121, 1/A-121 | usg_grid: main tee ROUNDUP(14.773/4.0)+1 = 5 x 38.833 = 194.16; cross tee ROUNDUP(38.833/1.333)+1 = 31 x 14.773 = 457.96; channel + angle molding 107.21 each</t>
+    <t xml:space="preserve">N/SHEET: 4/A-121, 1/A-121 | USG drywall suspension grid: main tee ROUNDUP(14.773/4.0)+1 = 5 x 38.833 = 194.16; cross tee ROUNDUP(38.833/1.333)+1 = 31 x 14.773 = 457.96; channel + angle molding 107.21 each</t>
   </si>
   <si>
     <t xml:space="preserve">USG drywall suspension cross tee DGLW424</t>
@@ -1180,7 +1180,7 @@
     <t xml:space="preserve">Additional head track at openings over 4'-0" wide</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: A-410, A-500 | Door 11 (W2-03): (4.0 + 2 x 0.667) x 1 = 5.33; Door 3 (C-H2a): (4.0 + 2 x 0.667) x 1 = 5.33</t>
+    <t xml:space="preserve">N/SHEET: A-500 | Door 11 (W2-03): (4.0 + 2 x 0.667) x 1 = 5.33; Door 3 (C-H2a): (4.0 + 2 x 0.667) x 1 = 5.33</t>
   </si>
   <si>
     <t xml:space="preserve">Stud reinforcement at MEP penetrations</t>
@@ -1189,7 +1189,7 @@
     <t xml:space="preserve">each</t>
   </si>
   <si>
-    <t xml:space="preserve">[RFI] N/SHEET: 6/A-410 | RFI: MEP sweep not registrable: mep.registro M-102 (page 48) vs A-101 (page 6) gave 20 / 14 matching wall segments (&lt; 25 required); the HVAC sheet is not used for geometric crossings ( rule). Ducts crossing the full-height type 2 / 5 / E walls must be counted from M-102 by the estimator. Delta: per duct crossing a stud wall: + MAX(1, ROUNDUP(duct width / 16")) stud reinforcement plates x stud rows (6/A-410 penetration details); plus 1 duct sleeve each</t>
+    <t xml:space="preserve">[RFI] N/SHEET: 6/A-410 | RFI: MEP sweep not registrable: the registration check of M-102 (page 48) vs A-101 (page 6) gave 20 / 14 matching wall segments (&lt; 25 required); the HVAC sheet is not used for geometric crossings (registration rule). Ducts crossing the full-height type 2 / 5 / E walls must be counted from M-102 by the estimator. Delta: per duct crossing a stud wall: + MAX(1, ROUNDUP(duct width / 16")) stud reinforcement plates x stud rows (6/A-410 penetration details); plus 1 duct sleeve each</t>
   </si>
   <si>
     <t xml:space="preserve">Extra framing - ATM recess (only what a detail prints at the recess; the wall stays in its type)</t>
@@ -1303,7 +1303,7 @@
     <t xml:space="preserve">RFI-ACC-stud-reinforcement-mep</t>
   </si>
   <si>
-    <t xml:space="preserve">stud reinforcement MEP: MEP sweep not registrable: mep.registro M-102 (page 48) vs A-101 (page 6) gave 20 / 14 matching wall segments (&lt; 25 required); the HVAC sheet is not used for geometric crossings (mep.py rule). Ducts crossing the full-height type 2 / 5 / E walls must be counted from M-102 by the estimator.</t>
+    <t xml:space="preserve">stud reinforcement MEP: MEP sweep not registrable: the registration check of M-102 (page 48) vs A-101 (page 6) gave 20 / 14 matching wall segments (&lt; 25 required); the HVAC sheet is not used for geometric crossings (registration rule). Ducts crossing the full-height type 2 / 5 / E walls must be counted from M-102 by the estimator.</t>
   </si>
   <si>
     <t xml:space="preserve">per duct crossing a stud wall: + MAX(1, ROUNDUP(duct width / 16")) stud reinforcement plates x stud rows (6/A-410 penetration details); plus 1 duct sleeve each</t>
@@ -1375,7 +1375,7 @@
     <t xml:space="preserve">CLOSED - Review Item rev3 (estimator decision 2026-10-26): type I WD-1 top = 15'-0" A.F.F. (6/A-226A; elevation bubble on 1/A-221 looks west at the type I face, verified).</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: 5/8" FRT plywood floor to 15'-0" = 3.31 LF x 15.0 = 49.65 SF; GWB 15'-0" to deck = 3.31 x 10.0 = 33.1 SF (2/A-221 studs UP TO DECK).</t>
+    <t xml:space="preserve">Applied (rev3 + rev5): type I 5/8" FRT plywood floor to 15'-0" (6/A-226A) = (C-I 2.31 + C-I-P.1 1.00 + end faces C-I-E1 / C-I-E2 1.21) 4.52 LF x 15.0 = 67.74 SF; GWB 15'-0" to deck 4.52 x 10.0 = 45.16 SF.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-09</t>
@@ -1600,7 +1600,7 @@
     <t xml:space="preserve">Grab &amp; Go header soffit (3/A-221): "T.O. WD-1 SEE ELEVATION" - top of WD-1 on the soffit east face not printed on A-226A / A-226B. Carried conservatively: 5/8" FRT plywood on the full east face (no GWB above WD-1).</t>
   </si>
   <si>
-    <t xml:space="preserve">Each 1 ft of face above T.O. WD-1 = 6.17 SF from 5/8" FRT plywood to 5/8" Type X GWB (full face 110.49 SF carried as plywood).</t>
+    <t xml:space="preserve">3/A-221 draws the 5/8" FRT plywood substrate full height and 5/8" GWB over it above T.O. WD-1: each 1 ft of face above T.O. WD-1 adds 6.17 SF of 5/8" Type X GWB (plywood 110.49 SF stays; GWB above WD-1 not carried until T.O. WD-1 is known).</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-35</t>
@@ -1609,7 +1609,7 @@
     <t xml:space="preserve">8/A-410 "METAL STUD/TRACK FIRE STOP AT CEILING LINE, TYP.": applied to every full-height wall with a ceiling on at least one face (1/A-121). audit rev4 (AUDITORIA_rev4/COMPARATIVA_AUDITORIA.xlsx row 7), rev5: carried; confirm with the GC that it is required at all of them.</t>
   </si>
   <si>
-    <t xml:space="preserve">Carried 230.14 LF track (3-5/8" 142.74 + 6" 87.40); if not required: - 230.14 LF.</t>
+    <t xml:space="preserve">Carried 264.21 LF track (3-5/8" 157.81 + 6" 106.40); if not required: - 264.21 LF.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-36</t>
@@ -1690,7 +1690,7 @@
     <t xml:space="preserve">Top / deflection and bottom track</t>
   </si>
   <si>
-    <t xml:space="preserve">Bottom track and top / deflection track = partition LF per type (A-101, A-221; 2/A-410, 3/A-410); + fire stop track at ceiling line 230.14 LF (8/A-410, RFI-35) and additional head track 10.67 LF (RFI-31); M-302 (p51) mention is plumbing expansion fittings</t>
+    <t xml:space="preserve">Bottom track and top / deflection track = partition LF per type (A-101, A-221; 2/A-410, 3/A-410); + fire stop track at ceiling line 264.21 LF (8/A-410, RFI-35) and additional head track 10.67 LF (RFI-31); M-302 (p51) mention is plumbing expansion fittings</t>
   </si>
   <si>
     <t xml:space="preserve">ALC-05</t>
@@ -1885,7 +1885,7 @@
     <t xml:space="preserve">reglas.py compuerta OK</t>
   </si>
   <si>
-    <t xml:space="preserve">{"canon": "c4d25e93c084c8a8c69060e0c1b08279a104b67302ddf031e4d013649cc8159a", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "35adec41fe38f2c867a49c924293d8f3b99a9904bed73e0f5d1a638ebec38a39", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
+    <t xml:space="preserve">{"canon": "daf95f92f470366cdce6f0acd1308b9bdb979b98e210e51b6fc2d13da1177060", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "876c39f2b252dd9003a84ea948ff0fee24c64c693064a34fa3fecfe1836c2fac", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
   </si>
 </sst>
 </file>
@@ -5699,7 +5699,7 @@
         <v>324</v>
       </c>
       <c r="C13" s="0" t="n">
-        <v>564.25</v>
+        <v>598.32</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -5707,18 +5707,18 @@
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">C13*D13</f>
-        <v>84.6375</v>
+        <v>89.748</v>
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">C13+E13</f>
-        <v>648.8875</v>
+        <v>688.068</v>
       </c>
       <c r="G13" s="0" t="s">
         <v>325</v>
       </c>
       <c r="H13" s="0" t="n">
         <f aca="false">ROUNDUP(F13/Inputs!$B$11,0)</f>
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I13" s="0" t="s">
         <v>342</v>

</xml_diff>